<commit_message>
new crime values, and draft scenario descriptions
</commit_message>
<xml_diff>
--- a/Data/Spreadsheets/CCJ_quantified_values.xlsx
+++ b/Data/Spreadsheets/CCJ_quantified_values.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11012"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11116"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/larapesceares/CCJ/Data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/larapesceares/CCJ/Data/Spreadsheets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{329D643F-A378-8141-B99C-D7C0E3165509}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBE83B2C-51D8-634F-B990-0A0F3FE41039}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="440" yWindow="3540" windowWidth="26780" windowHeight="12400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="394" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="442" uniqueCount="176">
   <si>
     <t>row_var</t>
   </si>
@@ -515,6 +515,54 @@
   </si>
   <si>
     <t>alt_wtp_freedom</t>
+  </si>
+  <si>
+    <t>crime_inc_soc</t>
+  </si>
+  <si>
+    <t>crime_inc_cost</t>
+  </si>
+  <si>
+    <t>crime_dec_soc</t>
+  </si>
+  <si>
+    <t>crime_dec_cost</t>
+  </si>
+  <si>
+    <t>Societal harm from increased crime due to detention</t>
+  </si>
+  <si>
+    <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC2835847/</t>
+  </si>
+  <si>
+    <t>Dobbie, Goldin &amp; Yang (2018)</t>
+  </si>
+  <si>
+    <t>https://www.nber.org/system/files/working_papers/w22511/w22511.pdf</t>
+  </si>
+  <si>
+    <t>Government CJS costs from increased crime</t>
+  </si>
+  <si>
+    <t>Societal benefits from decreased crime</t>
+  </si>
+  <si>
+    <t>Government CJS cost savings from decreased crime</t>
+  </si>
+  <si>
+    <t>McCollister et al. (2010)</t>
+  </si>
+  <si>
+    <t>felony: 59,900; misdemeanor: 80</t>
+  </si>
+  <si>
+    <t>Upper CI (+14 p.p.)</t>
+  </si>
+  <si>
+    <t>felony: 10,200; misdemeanor: 4,600</t>
+  </si>
+  <si>
+    <t>Lower CI (–4 p.p.)</t>
   </si>
 </sst>
 </file>
@@ -614,7 +662,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -631,10 +679,8 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -942,7 +988,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{018C5E1B-70FC-CE48-BD0C-84D5CA275194}">
-  <dimension ref="A1:T14"/>
+  <dimension ref="A1:T19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.33203125" bestFit="1" customWidth="1"/>
@@ -1117,53 +1163,53 @@
         <v>106</v>
       </c>
     </row>
-    <row r="5" spans="1:20" s="14" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="14" t="s">
+    <row r="5" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="B5" t="s">
         <v>134</v>
       </c>
-      <c r="C5" s="15" t="s">
+      <c r="C5" s="14" t="s">
         <v>156</v>
       </c>
-      <c r="D5" s="14">
+      <c r="D5">
         <v>1</v>
       </c>
-      <c r="E5" s="14" t="s">
+      <c r="E5" t="s">
         <v>137</v>
       </c>
-      <c r="F5" s="14" t="s">
+      <c r="F5" t="s">
         <v>35</v>
       </c>
-      <c r="G5" s="14">
+      <c r="G5">
         <v>2023</v>
       </c>
-      <c r="H5" s="14" t="s">
+      <c r="H5" t="s">
         <v>151</v>
       </c>
-      <c r="I5" s="16">
+      <c r="I5" s="3">
         <v>294728</v>
       </c>
-      <c r="J5" s="16">
+      <c r="J5" s="3">
         <v>100000</v>
       </c>
-      <c r="K5" s="16">
+      <c r="K5" s="3">
         <v>300000</v>
       </c>
-      <c r="L5" s="14" t="s">
+      <c r="L5" t="s">
         <v>152</v>
       </c>
-      <c r="M5" s="17" t="s">
+      <c r="M5" s="15" t="s">
         <v>147</v>
       </c>
-      <c r="N5" s="14" t="s">
+      <c r="N5" t="s">
         <v>148</v>
       </c>
-      <c r="O5" s="14" t="s">
+      <c r="O5" t="s">
         <v>146</v>
       </c>
-      <c r="P5" s="14" t="s">
+      <c r="P5" t="s">
         <v>149</v>
       </c>
     </row>
@@ -1487,6 +1533,194 @@
       </c>
       <c r="N14" t="s">
         <v>44</v>
+      </c>
+    </row>
+    <row r="16" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>160</v>
+      </c>
+      <c r="B16" t="s">
+        <v>134</v>
+      </c>
+      <c r="C16" t="s">
+        <v>164</v>
+      </c>
+      <c r="D16">
+        <v>2</v>
+      </c>
+      <c r="E16" t="s">
+        <v>137</v>
+      </c>
+      <c r="F16" t="s">
+        <v>35</v>
+      </c>
+      <c r="G16">
+        <v>2008</v>
+      </c>
+      <c r="H16" t="s">
+        <v>172</v>
+      </c>
+      <c r="I16">
+        <v>-5900</v>
+      </c>
+      <c r="K16" t="s">
+        <v>173</v>
+      </c>
+      <c r="L16" t="s">
+        <v>171</v>
+      </c>
+      <c r="M16" t="s">
+        <v>165</v>
+      </c>
+      <c r="N16" t="s">
+        <v>166</v>
+      </c>
+      <c r="O16" t="s">
+        <v>167</v>
+      </c>
+      <c r="P16" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>161</v>
+      </c>
+      <c r="B17" t="s">
+        <v>136</v>
+      </c>
+      <c r="C17" t="s">
+        <v>168</v>
+      </c>
+      <c r="D17">
+        <v>2</v>
+      </c>
+      <c r="E17" t="s">
+        <v>137</v>
+      </c>
+      <c r="F17" t="s">
+        <v>115</v>
+      </c>
+      <c r="G17">
+        <v>2008</v>
+      </c>
+      <c r="H17" t="s">
+        <v>174</v>
+      </c>
+      <c r="I17">
+        <v>1200</v>
+      </c>
+      <c r="K17" t="s">
+        <v>173</v>
+      </c>
+      <c r="L17" t="s">
+        <v>171</v>
+      </c>
+      <c r="M17" t="s">
+        <v>165</v>
+      </c>
+      <c r="N17" t="s">
+        <v>166</v>
+      </c>
+      <c r="O17" t="s">
+        <v>167</v>
+      </c>
+      <c r="P17" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>162</v>
+      </c>
+      <c r="B18" t="s">
+        <v>134</v>
+      </c>
+      <c r="C18" t="s">
+        <v>169</v>
+      </c>
+      <c r="D18">
+        <v>2</v>
+      </c>
+      <c r="E18" t="s">
+        <v>137</v>
+      </c>
+      <c r="F18" t="s">
+        <v>115</v>
+      </c>
+      <c r="G18">
+        <v>2008</v>
+      </c>
+      <c r="H18" t="s">
+        <v>172</v>
+      </c>
+      <c r="I18">
+        <v>1700</v>
+      </c>
+      <c r="K18" t="s">
+        <v>175</v>
+      </c>
+      <c r="L18" t="s">
+        <v>171</v>
+      </c>
+      <c r="M18" t="s">
+        <v>165</v>
+      </c>
+      <c r="N18" t="s">
+        <v>166</v>
+      </c>
+      <c r="O18" t="s">
+        <v>167</v>
+      </c>
+      <c r="P18" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>163</v>
+      </c>
+      <c r="B19" t="s">
+        <v>136</v>
+      </c>
+      <c r="C19" t="s">
+        <v>170</v>
+      </c>
+      <c r="D19">
+        <v>2</v>
+      </c>
+      <c r="E19" t="s">
+        <v>137</v>
+      </c>
+      <c r="F19" t="s">
+        <v>35</v>
+      </c>
+      <c r="G19">
+        <v>2008</v>
+      </c>
+      <c r="H19" t="s">
+        <v>174</v>
+      </c>
+      <c r="I19">
+        <v>-340</v>
+      </c>
+      <c r="K19" t="s">
+        <v>175</v>
+      </c>
+      <c r="L19" t="s">
+        <v>171</v>
+      </c>
+      <c r="M19" t="s">
+        <v>165</v>
+      </c>
+      <c r="N19" t="s">
+        <v>166</v>
+      </c>
+      <c r="O19" t="s">
+        <v>167</v>
+      </c>
+      <c r="P19" t="s">
+        <v>167</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
new descriptions for scenerios, no crime effect scenerios now
</commit_message>
<xml_diff>
--- a/Data/Spreadsheets/CCJ_quantified_values.xlsx
+++ b/Data/Spreadsheets/CCJ_quantified_values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/larapesceares/CCJ/Data/Spreadsheets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBE83B2C-51D8-634F-B990-0A0F3FE41039}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4FF3163-148D-784E-B9C8-C23F19AA8B08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="440" yWindow="3540" windowWidth="26780" windowHeight="12400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="3420" windowWidth="24920" windowHeight="15020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Baseline components " sheetId="4" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="442" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="444" uniqueCount="176">
   <si>
     <t>row_var</t>
   </si>
@@ -988,7 +988,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{018C5E1B-70FC-CE48-BD0C-84D5CA275194}">
-  <dimension ref="A1:T19"/>
+  <dimension ref="A1:T23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.33203125" bestFit="1" customWidth="1"/>
@@ -1723,12 +1723,23 @@
         <v>167</v>
       </c>
     </row>
+    <row r="22" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="H22" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="H23" t="s">
+        <v>174</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="N9" r:id="rId1" xr:uid="{126C1809-D3C8-9244-9EA2-45648641ED16}"/>
     <hyperlink ref="O6" r:id="rId2" xr:uid="{A36DD19A-6484-BA44-A71E-581B1317BD8B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 

</xml_diff>